<commit_message>
Development of F. Developer logging & system documentation
</commit_message>
<xml_diff>
--- a/docs/Phase 3 Enhancements or Feedback/ATS App - Phase wise Task Items.xlsx
+++ b/docs/Phase 3 Enhancements or Feedback/ATS App - Phase wise Task Items.xlsx
@@ -28,7 +28,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Phase 3 OLd V1'!$C$1:$C$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phase 3 Enh - Do Now'!$A$1:$J$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Phase 3 Enh - Phase 4'!$A$1:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Phase 3 Enh - Phase 4'!$A$1:$J$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Phase 4 - Updated'!$A$1:$J$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Phase 2 Feedback- Iteration 3'!$A$1:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Phase 2 Feedback- Iteration1'!$C$1:$K$1</definedName>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4784" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4789" uniqueCount="1173">
   <si>
     <t>Task</t>
   </si>
@@ -3701,7 +3701,8 @@
   </si>
   <si>
     <t>RT §5 fresher rating.
-[15 Oct] Experience band, budget and education checks. In commit 4227049 (14 Oct). Live only with SCREENING_V2=true in the backend env. Where: docs/changelog/CHANGES-2026-10-14-strict-jd-filtering.md</t>
+[15 Oct] Experience band, budget and education checks. In commit 4227049 (14 Oct). Live only with SCREENING_V2=true in the backend env. Where: docs/changelog/CHANGES-2026-10-14-strict-jd-filtering.md
+[19 Oct] Fix: a line added on 14 Oct sat in the wrong handler, so viewing an MRF request (GET /api/mrf/:id) always failed and editing a budget did not refresh JD results. Fixed with section E. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
   </si>
   <si>
     <t>N09 · JD - ranking</t>
@@ -3981,7 +3982,8 @@
   <si>
     <t>Our item; our bug #5. pipeline.service.js:709.
 [15 Oct] Parked 15 Oct. Plan ready, about 11 h; needs a drawer mockup. Decision pending: Excel scores read-only in Search Candidate edit (recommended).
-[16 Oct] Built: every round keeps its own scores (Zeko scores and report, Evalground report link, each interviewer's average /5 and verdict) and a read-only "Uploaded scores (from Excel)" card. Fixed: the HR card showed Functional's scores. Layout: per round, no summary strip. Unit tests pass; screen check pending (needs a login). Not yet on staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
+[16 Oct] Built: every round keeps its own scores (Zeko scores and report, Evalground report link, each interviewer's average /5 and verdict) and a read-only "Uploaded scores (from Excel)" card. Fixed: the HR card showed Functional's scores. Layout: per round, no summary strip. Unit tests pass; screen check pending (needs a login). Not yet on staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
+[19 Oct] Tested on staging data: a passed Zeko round keeps its own scores; the "Uploaded scores" card shows (e2e/section-d.spec.js pass). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
   </si>
   <si>
     <t>N29 · Candidate data sync</t>
@@ -3994,7 +3996,8 @@
   <si>
     <t>Our bug #2. candidate.service.js:517-564.
 [15 Oct] Parked 15 Oct. Plan ready, about 15 h. Decision pending: rebuild the search profile after an edit (one AI call per edit; recommended yes).
-[16 Oct] Built: name/email edits reach the pipeline and its emails from every writer (Search Candidate, missing-details form, uploads, Outlook); read-only Pipeline scores in Search Candidate; the edit form saves only changed fields; editing is staff only. Integration test 5/5 on staging; backfill applied on staging (2 rows). Audit: docs/reference/candidate-data-copies.md. Screen check pending. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
+[16 Oct] Built: name/email edits reach the pipeline and its emails from every writer (Search Candidate, missing-details form, uploads, Outlook); read-only Pipeline scores in Search Candidate; the edit form saves only changed fields; editing is staff only. Integration test 5/5 on staging; backfill applied on staging (2 rows). Audit: docs/reference/candidate-data-copies.md. Screen check pending. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
+[19 Oct] Tested on staging data: integration test 6/6 (incl. an old missing-details link after an email edit); Search Candidate pipeline scores pass on screen. Open: the link after an upload merge (needs a real upload). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
   </si>
   <si>
     <t>N30 · Pipeline popup crash</t>
@@ -4030,482 +4033,467 @@
   </si>
   <si>
     <t>Our bug #4.
-[15 Oct] Week 1. Built and tested locally; not yet on staging (dev &gt; staging, production once at the end). Where: docs/changelog/CHANGES-2026-10-14-phase3-week1.md
-[16 Oct ]- TESTING RESULT- all the instances haven't been covered as I can see the staging a and staging b data in the MRF VIew/edit page.
-[16 Oct] Reopen fixed in code: the MRF page, the public approval page and the MRF export show names from the current approver list (by email), so old MRFs show real names too. Staging data: the approver list was overwritten by the N16 integration test's clean-up (it still holds the test values); restore pending. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
-  </si>
-  <si>
-    <t>N33 · Skip guard</t>
-  </si>
-  <si>
-    <t>Today: The skip-stage API doesn't check that the stage is optional, so any staff user could skip any stage.
-Change: Server-side check: only optional stages can be skipped.
-Done when: Skipping a mandatory stage through the API is refused.</t>
-  </si>
-  <si>
-    <t>Found in code review. pipeline.service.js:1090.
-[15 Oct] Week 1. The server refuses skipping a mandatory stage. Built and tested locally; not yet on staging (dev &gt; staging, production once at the end). Where: docs/changelog/CHANGES-2026-10-14-phase3-week1.md</t>
-  </si>
-  <si>
-    <t>N34 · Date format</t>
-  </si>
-  <si>
-    <t>Today: Dates appear in about 13 different formats, some depending on the browser's locale.
-Change: One shared date / time helper (IST) used across the app.
-Done when: Every date on screen follows the same format.</t>
-  </si>
-  <si>
-    <t>Our item.
-[15 Oct] Parked 15 Oct. Plan ready, about 7 h. The shared helper frontend/src/utils/dateFormat.js was started in week 1.
-[16 Oct] Built: one IST format on ~20 screens and in all emails (07 Oct 2026, 4:30 PM IST); fixed the new-MRF email date that followed the server's locale. Unit tests pass; screen check pending. Not yet on staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
-  </si>
-  <si>
-    <t>E. CEO clarity, dashboard &amp; analytics</t>
-  </si>
-  <si>
-    <t>N35 · Labels &amp; legends</t>
-  </si>
-  <si>
-    <t>Today: The CEO couldn't tell what pipeline columns and statuses mean. "Invited" actually means the Zeko link was sent and "In progress" means not yet invited (explained the other way round in the demo). The board doesn't show whether an Evalground test was sent.
-Change: Clear stage / status names and a legend on the pipeline board; "Test sent - due date / Overdue" on Evalground cards; review other unclear labels (screening match chips, upload job statuses) and add tooltips.
-Done when: Someone new can read the board without explanation.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 3 Enh. rows 3-4).</t>
-  </si>
-  <si>
-    <t>N36 · Dashboard fixes</t>
-  </si>
-  <si>
-    <t>Today: Trends and top roles use only the newest 200 candidates; Shortlisted / Hired counts use old status values; Upcoming Interviews shows only Zeko windows (no Teams interviews) and opens Analytics; recent uploads don't open the candidate; the role filter uses the candidate's typed "Position Applied".
-Change: Server-side totals; counts aligned with pipeline statuses; Teams interviews included; rows open the right candidate; role filter by MRF; clear shortlist-rate definition.
-Done when: Dashboard numbers match Analytics and Search Candidate for the same period.</t>
-  </si>
-  <si>
-    <t>Our #61; 10 Sep dashboard-numbers item.</t>
-  </si>
-  <si>
-    <t>N37 · Raw vs qualified (interim)</t>
-  </si>
-  <si>
-    <t>Today: There is no view of raw vs qualified candidate numbers.
-Change: Two numbers from existing data: raw (all candidates in the period) and qualified (completed the details form or replied). Definition agreed with Chhaya first.
-Done when: Both numbers show on the dashboard, with the definition in a tooltip.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 3 Enh. row 2). The stored status is Responded status &amp; source marker (P01).</t>
-  </si>
-  <si>
-    <t>N38 · Recency filter</t>
-  </si>
-  <si>
-    <t>Today: Screening can't be limited to recent candidates, and the ranking doesn't use dates.
-Change: "Added in" filter: last 7 / 10 / 15 days, 1 month, 3 months.
-Done when: The filter works in both keyword and JD screening.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 4 sheet row 84). Dates in the ranking are Scoring weights &amp; recency (L01).</t>
-  </si>
-  <si>
-    <t>N39 · Analytics - Positions tab</t>
-  </si>
-  <si>
-    <t>Today: Analytics shows one MRF at a time; there is no cross-position view, no open-to-close journey and no joining ratio.
-Change: New tab with one row per MRF: opened, days open, shortlisted, candidates per stage, offers, joined, closed and reason; hiring-to-joining ratio; per-role "Moved Forward".
-Done when: Every position's status is visible on one screen.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 3 Enh. row 5); Anuj in the demo.</t>
-  </si>
-  <si>
-    <t>F. Developer logging &amp; system documentation</t>
-  </si>
-  <si>
-    <t>N42 · Developer logging &amp; error tracing</t>
-  </si>
-  <si>
-    <t>Today: Developers hear about problems from HR. Logs are files on the server, and nothing ties an HR report to a log line. Scheduled-job failures and crashes are only logged, and browser errors aren't captured.
-Change: A reference ID on every request, shown in error messages ("ref: AB12CD"); logging of calls to Graph, Zeko, the AI service and Cohere; alerts on job failures and crashes; browser error capture; an admin "Logs &amp; errors" page searchable by reference, user and time; a deep health check. Personal data is masked in all logs.
-Done when: HR quotes the error reference shown on screen, and a developer finds the full trail in under 2 minutes without logging in to the server.</t>
-  </si>
-  <si>
-    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.</t>
-  </si>
-  <si>
-    <t>N43 · System documentation &amp; development history</t>
-  </si>
-  <si>
-    <t>Today: Knowledge is spread across 50+ feature plans, RCAs and changelogs. Nothing describes how the system works as a whole, what has been built since January, or how to handle common incidents.
-Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it.
-Done when: A developer new to the project can set up, find any module, handle a common incident, and see what was built, when and why, from these docs alone.</t>
-  </si>
-  <si>
-    <t>Week 4-5</t>
-  </si>
-  <si>
-    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.</t>
-  </si>
-  <si>
-    <t>G. Housekeeping (no code)</t>
-  </si>
-  <si>
-    <t>N40 · Housekeeping</t>
-  </si>
-  <si>
-    <t>Today: Stale / test MRFs (e.g. Business Development Services, T Snap Project One) show as open; Samriddhi is tagged to the wrong JD; HRD (Susmita, Subhajit) run some hiring outside the ATS.
-Change: Close the stale MRFs with a reason; close Samriddhi's wrong journey; create ATS logins with upload access for Susmita and Subhajit (role and modules set by the admin).
-Done when: The open-positions list is accurate and HRD candidates are entered in the ATS.</t>
-  </si>
-  <si>
-    <t>Demo 28 Sep. Admin action.
-[15 Oct] Admin action, not done yet. Steps in docs/changelog/CHANGES-2026-10-14-phase3-week1.md (release step 9).</t>
-  </si>
-  <si>
-    <t>H. To brainstorm later</t>
-  </si>
-  <si>
-    <t>N41 · Upload speed</t>
-  </si>
-  <si>
-    <t>Today: RT reports that uploads take too long; each resume or Excel row is parsed by AI one at a time, followed by more AI work per candidate.
-Change: To be decided in a separate brainstorm once all other Do Now items are closed.
-Done when: -</t>
-  </si>
-  <si>
-    <t>Brainstorm later</t>
-  </si>
-  <si>
-    <t>After other items</t>
-  </si>
-  <si>
-    <t>RT "Matching &amp; score analysis takes too long to upload".</t>
-  </si>
-  <si>
-    <t>Search, scoring &amp; candidate movement</t>
-  </si>
-  <si>
-    <t>L01 · Scoring weights &amp; recency</t>
-  </si>
-  <si>
-    <t>Today: After JD - skill gate through JD - ranking (N07–N09), ranking among qualified candidates uses fixed weights and ignores when a candidate applied.
-Change: Re-tune weights and score bands with RT; rank recent applicants higher.
-Done when: RT agrees with the ranking on their sample JDs.</t>
-  </si>
-  <si>
-    <t>RT §5; CEO (Phase 4 sheet row 84).</t>
-  </si>
-  <si>
-    <t>L02 · Move / re-tag candidate</t>
-  </si>
-  <si>
-    <t>Today: A candidate already tagged to one JD can't be moved to another; a wrong tag can only be closed; tags always start at the first stage.
-Change: Move a candidate to another JD with a chosen landing stage (history kept); remove a wrong tag.
-Done when: A final-round candidate can move to a new role at a chosen stage without extra emails.</t>
-  </si>
-  <si>
-    <t>RT §6.2. Needs RT's decision on where a moved candidate lands.</t>
-  </si>
-  <si>
-    <t>L03 · Flexible stages</t>
-  </si>
-  <si>
-    <t>Today: The pipeline moves forward one stage at a time; only Tech 3 and the Client round can be skipped; a skipped stage can never be done later.
-Change: Authorized users can skip stages (e.g. HR Screening -&gt; Evalground, HR Screening -&gt; Functional, Assessment -&gt; CEO round) and re-open or complete a skipped stage later (walk-in: Tech 1 first, Evalground at the weekend). Evalground import matches candidates at any stage; candidates get no duplicate emails.
-Done when: The walk-in example runs end to end with correct emails and history.</t>
-  </si>
-  <si>
-    <t>RT §7. Needs written answers: who may skip, and what the candidate is told.</t>
-  </si>
-  <si>
-    <t>MRF &amp; pipeline hygiene</t>
-  </si>
-  <si>
-    <t>L04 · MRF Hold</t>
-  </si>
-  <si>
-    <t>Today: Approvers can only approve or reject an MRF.
-Change: Hold option (with a note and hold-until date) at approval; on that date the approver is reminded with Approve / Reject / Hold further; held MRFs appear as open nowhere.
-Done when: A held MRF re-prompts its approver on the hold-until date.</t>
-  </si>
-  <si>
-    <t>RT §1.</t>
-  </si>
-  <si>
-    <t>L05 · Drop-out rules</t>
-  </si>
-  <si>
-    <t>Today: Candidates who never take a Zeko test or respond stay in the pipeline indefinitely and clutter the columns.
-Change: Per-stage reminder and timeout rules; auto-close as "Unresponsive" after the timeout; settings to tune them.
-Done when: Non-responders leave the board automatically after the set time.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 4 sheet row 85). Needs RT sign-off (current rule: recruiter decides).</t>
-  </si>
-  <si>
-    <t>Analytics &amp; JD records</t>
-  </si>
-  <si>
-    <t>L06 · Analytics - date range &amp; Total Applied</t>
-  </si>
-  <si>
-    <t>Today: Analytics uses fixed windows, and "Total Applied" per role can't be counted without JD tags.
-Change: Presets (30 / 60 / 90 / 365 days, all) plus a custom date picker applied to every tile; per-role "Total Applied" from the JD tags (JD tagging on upload (N13–N15)).
-Done when: Every Analytics number follows the chosen range.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 3 Enh. row 5); 10 Sep review.</t>
-  </si>
-  <si>
-    <t>L07 · Editable JD label (no MRF)</t>
-  </si>
-  <si>
-    <t>Today: JDs without an MRF have no date or label to tell versions apart.
-Change: Recruiter-editable date / label on such JDs, shown next to the JD name.
-Done when: RT can mark the latest version of a JD that has no MRF.</t>
-  </si>
-  <si>
-    <t>RT §3 (second half).</t>
-  </si>
-  <si>
-    <t>Other Bugs</t>
-  </si>
-  <si>
-    <t>Adhoc links for all forms</t>
-  </si>
-  <si>
-    <t>If Recruiter wants to access some links, right now, they are not accessible easily. Let's say I have sent a link to interviewer post interview, I can't find the link form the app easily. There are lot more forms and lot more links. If we can arrange those links in some page, it would make things easier for recruiter for fetch any link</t>
-  </si>
-  <si>
-    <t>HR Manual Upload &amp; Vendor Manual Upload</t>
-  </si>
-  <si>
-    <t>If there is any duplicate, right now,REVIEW is showing what is the current user name and his/her resume instead of a pure comparison of what data has been there already vs what is new one and what changed since last resume etc.</t>
-  </si>
-  <si>
-    <t>HR Manual Upload - User Profile redirect</t>
-  </si>
-  <si>
-    <t>In the resume uploaded by HR, if user wants to check the candidate details in detail, they don't have the option to redirect the user to the candidate profile view page.</t>
-  </si>
-  <si>
-    <t>Candidate Screening - Hidden by system data</t>
-  </si>
-  <si>
-    <t>For example - "8 recently rejected for this role · 3 meet education, budget and experience · of those, 0 have all 7 mandatory skills
-" for this case, if I wish to see the data, there is no such option exist now.</t>
-  </si>
-  <si>
-    <t>s</t>
-  </si>
-  <si>
-    <t>Vendor 2 - C2C Vendor (on hold)</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. NULL vendor_type = placement backward-compatible</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months.</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Keeps shared tracking/status steps single-sourced</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Rate/Duration required for C2C optional for placement</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Shared engine reused - not a fork of the 1724-line runBatchParsing</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Flags already_in_main_pool - never auto-merges/rejects</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Name collision in C2C is expected not an error</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Review never vendor-accessible</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Never mutate the raw Name field</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Education + stability weights zeroed for C2C</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Reuses existing premium upload components</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. No UNION logic needed in controller</t>
-  </si>
-  <si>
-    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Proves the shared engine was not regressed</t>
-  </si>
-  <si>
-    <t>MS Access (R&amp;D / export)</t>
-  </si>
-  <si>
-    <t>Other Phase 4 items</t>
-  </si>
-  <si>
-    <t>P01 · Responded status &amp; source marker</t>
-  </si>
-  <si>
-    <t>Today: Nothing records whether a candidate responded to outreach or is an old database record, so search can't prefer active applicants.
-Change: Store the responded status and source (new applicant vs old database); rank late responders lower; "Responders only" option in search; the Raw vs qualified (interim) (N37) counts switch to the stored status.
-Done when: Search can be limited to responders, and each card shows "Responded" or "From old database".</t>
-  </si>
-  <si>
-    <t>CEO (Phase 3 Enh. row 2; Phase 4 sheet row 83).</t>
-  </si>
-  <si>
-    <t>P02 · Hiring-manager status email</t>
-  </si>
-  <si>
-    <t>Today: RT sends daily / weekly position updates to hiring managers by hand.
-Change: Automatic daily or weekly email to each hiring manager about their open positions (candidates per stage, upcoming interviews, offers); schedule set in Settings.
-Done when: Hiring managers receive it without RT's involvement.</t>
-  </si>
-  <si>
-    <t>Anuj in the demo; our #71.</t>
-  </si>
-  <si>
-    <t>P03 · Hiring-manager read-only role</t>
-  </si>
-  <si>
-    <t>Today: Hiring managers have no ATS login.
-Change: A read-only role that sees only the hiring manager's own positions (pipeline and analytics).
-Done when: A hiring manager logs in and sees only their positions, with no edit actions.</t>
-  </si>
-  <si>
-    <t>CEO (Phase 4 sheet row 86). Hiring-manager status email (P02) covers the status need first.</t>
-  </si>
-  <si>
-    <t>P04 · SMS / WhatsApp reminders</t>
-  </si>
-  <si>
-    <t>Today: The ATS can only send email.
-Change: Interview reminders by SMS / WhatsApp through a provider, using the phone captured in Candidate phone &amp; interview reminders (N22).
-Done when: A scheduled interview triggers an SMS / WhatsApp reminder.</t>
-  </si>
-  <si>
-    <t>RT §9. Needs a provider.</t>
-  </si>
-  <si>
-    <t>P05 · Prompt configuration</t>
-  </si>
-  <si>
-    <t>Today: All six AI prompts (JD parse, resume parse, two insight prompts, two Evalground prompts) are hard-coded.
-Change: Admin screen to view and edit prompts, with versioning, reset to default and a test run.
-Done when: A prompt can be changed and rolled back without a deployment.</t>
-  </si>
-  <si>
-    <t>Our list.</t>
-  </si>
-  <si>
-    <t>P06 · Reminder settings in one place</t>
-  </si>
-  <si>
-    <t>Today: Settings &gt; Reminder Settings covers only three reminder types; interview, occurrence, document and assessment reminders are set elsewhere or in server config.
-Change: Bring every reminder's on/off switch, timing and limits under one Settings section.
-Done when: All reminders can be tuned from Settings.</t>
-  </si>
-  <si>
-    <t>P07 · Website candidates report</t>
-  </si>
-  <si>
-    <t>Today: Website applications reach the ATS through the recruitment mailbox but aren't marked as website-sourced, and RT has no daily report of them.
-Change: Store a permanent intake source on each candidate; daily 8 AM email to RT with the current month's website candidates as Excel; on the 1st, a second email with the previous month's summary.
-Done when: RT receives both emails on schedule.</t>
-  </si>
-  <si>
-    <t>Our list (Website Data Update; Website Integration).</t>
-  </si>
-  <si>
-    <t>P08 · Captcha on public MRF form</t>
-  </si>
-  <si>
-    <t>Today: Captcha protects the login pages, but the public MRF submission form has no captcha or rate limit.
-Change: Add captcha and a rate limit to the public MRF form.
-Done when: Automated submissions are blocked.</t>
-  </si>
-  <si>
-    <t>Our list (Captcha).</t>
-  </si>
-  <si>
-    <t>P09 · Zeko 90-day re-interview check</t>
-  </si>
-  <si>
-    <t>Today: Nothing stops a Zeko interview being sent again to a candidate interviewed in the last 90 days.
-Change: Warn or block re-sending within 90 days and reuse the previous result; investigate whether Zeko's API allows archiving or deleting old interview data.
-Done when: Re-sending within 90 days shows a warning with the previous result.</t>
-  </si>
-  <si>
-    <t>Our list (R&amp;D). Hours exclude the Zeko API research.</t>
-  </si>
-  <si>
-    <t>P10 · Admin Config UI polish</t>
-  </si>
-  <si>
-    <t>Today: Admins can edit stages, outcomes and reasons, but there is no hard delete, no in-use check when deactivating outcomes or reasons, no audit of config changes, and new custom interview stages get no scheduling or scorecards.
-Change: Add those four.
-Done when: Config changes are logged and can't break candidates mid-stage.</t>
-  </si>
-  <si>
-    <t>P11 · Excel scores to round scorecards</t>
-  </si>
-  <si>
-    <t>Today: Interview scores in Excel uploads are stored on the candidate record, not in the round scorecards the pipeline uses (Scores in the pipeline drawer (N28) only displays them).
-Change: Import them into the matching round's scorecard.
-Done when: Uploaded scores appear as real round scores.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CEO (Phase 3 Enh. rows 3-4).
-[19 Oct] Built: plain card labels (Not yet invited / Zeko link sent / Not yet scheduled / Awaiting action / Awaiting decision / Test not sent / Test sent · due &lt;date&gt; / Test overdue) with hover text; a "What do these mean?" legend on the board; stage meanings on column headers; clearer labels and tooltips on Screening chips, upload statuses, MRF badges and the Vendor dashboard. Tested on staging data: labels, legend and assessment cards pass (e2e/section-e.spec.js). Final wording to confirm with RT. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our #61; 10 Sep dashboard-numbers item.
-[19 Oct] Built: dashboard counts every candidate on the server (no 200 cap); Shortlisted = in the pipeline now, Hired = the Analytics rule; working MRF filter; Zeko + Teams in Upcoming Interviews; rows open the candidate; "Definitions updated" note. Tested on staging data: matches Analytics for 7/30/90 days and per MRF (check-dashboard-vs-analytics.mjs all OK); filters and links pass on screen. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CEO (Phase 3 Enh. row 2). The stored status is Responded status &amp; source marker (P01).
-[19 Oct] On hold until Chhaya agrees the definition. Proposed: raw = candidates added in the period; qualified = those who completed the details form or replied by email. Totals only until JD tagging (N13). About 6 h once agreed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CEO (Phase 4 sheet row 84). Dates in the ranking are Scoring weights &amp; recency (L01).
-[19 Oct] Built: "Added within" 7 / 10 / 15 days, 1 month, 3 months on Keyword and JD screening; the JD CSV follows the filter. Tested on staging data: JD integration 13/13 incl. the 15-day case; both filters pass on screen. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CEO (Phase 3 Enh. row 5); Anuj in the demo.
-[19 Oct] Built: Analytics "Positions" tab, one row per MRF (opened, days open, per-stage counts, offers, joined, joining ratio, closure reason), sortable, CSV, a row opens that MRF's funnel. Tested on staging data: rows, sort, filter, CSV and row-to-funnel pass. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our item; our bug #5. pipeline.service.js:709.
-[15 Oct] Parked 15 Oct. Plan ready, about 11 h; needs a drawer mockup. Decision pending: Excel scores read-only in Search Candidate edit (recommended).
-[16 Oct] Built: every round keeps its own scores (Zeko scores and report, Evalground report link, each interviewer's average /5 and verdict) and a read-only "Uploaded scores (from Excel)" card. Fixed: the HR card showed Functional's scores. Layout: per round, no summary strip. Unit tests pass; screen check pending (needs a login). Not yet on staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
-[19 Oct] Tested on staging data: a passed Zeko round keeps its own scores; the "Uploaded scores" card shows (e2e/section-d.spec.js pass). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our bug #2. candidate.service.js:517-564.
-[15 Oct] Parked 15 Oct. Plan ready, about 15 h. Decision pending: rebuild the search profile after an edit (one AI call per edit; recommended yes).
-[16 Oct] Built: name/email edits reach the pipeline and its emails from every writer (Search Candidate, missing-details form, uploads, Outlook); read-only Pipeline scores in Search Candidate; the edit form saves only changed fields; editing is staff only. Integration test 5/5 on staging; backfill applied on staging (2 rows). Audit: docs/reference/candidate-data-copies.md. Screen check pending. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
-[19 Oct] Tested on staging data: integration test 6/6 (incl. an old missing-details link after an email edit); Search Candidate pipeline scores pass on screen. Open: the link after an upload merge (needs a real upload). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Our bug #4.
 [15 Oct] Week 1. Built and tested locally; not yet on staging (dev &gt; staging, production once at the end). Where: docs/changelog/CHANGES-2026-10-14-phase3-week1.md
 [16 Oct ]- TESTING RESULT- all the instances haven't been covered as I can see the staging a and staging b data in the MRF VIew/edit page.
 [16 Oct] Reopen fixed in code: the MRF page, the public approval page and the MRF export show names from the current approver list (by email), so old MRFs show real names too. Staging data: the approver list was overwritten by the N16 integration test's clean-up (it still holds the test values); restore pending. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
 [19 Oct] The approver test still waits for the staging approver list to be restored. Note: 3 staging email settings (mrfApproval, mrfSubmitHrNotify, mrfOutcome) still list saukumar@; harmless on staging (mail is redirected to the test inboxes); check the production values before the final release.</t>
   </si>
   <si>
-    <t xml:space="preserve">Our item.
+    <t>N33 · Skip guard</t>
+  </si>
+  <si>
+    <t>Today: The skip-stage API doesn't check that the stage is optional, so any staff user could skip any stage.
+Change: Server-side check: only optional stages can be skipped.
+Done when: Skipping a mandatory stage through the API is refused.</t>
+  </si>
+  <si>
+    <t>Found in code review. pipeline.service.js:1090.
+[15 Oct] Week 1. The server refuses skipping a mandatory stage. Built and tested locally; not yet on staging (dev &gt; staging, production once at the end). Where: docs/changelog/CHANGES-2026-10-14-phase3-week1.md</t>
+  </si>
+  <si>
+    <t>N34 · Date format</t>
+  </si>
+  <si>
+    <t>Today: Dates appear in about 13 different formats, some depending on the browser's locale.
+Change: One shared date / time helper (IST) used across the app.
+Done when: Every date on screen follows the same format.</t>
+  </si>
+  <si>
+    <t>Our item.
 [15 Oct] Parked 15 Oct. Plan ready, about 7 h. The shared helper frontend/src/utils/dateFormat.js was started in week 1.
 [16 Oct] Built: one IST format on ~20 screens and in all emails (07 Oct 2026, 4:30 PM IST); fixed the new-MRF email date that followed the server's locale. Unit tests pass; screen check pending. Not yet on staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md
 [19 Oct] Tested on staging data: no locale-dependent dates on the 6 main pages with an en-US browser (e2e/section-d.spec.js pass). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-16-phase3-section-d.md</t>
   </si>
   <si>
-    <t xml:space="preserve">RT §5 fresher rating.
-[15 Oct] Experience band, budget and education checks. In commit 4227049 (14 Oct). Live only with SCREENING_V2=true in the backend env. Where: docs/changelog/CHANGES-2026-10-14-strict-jd-filtering.md
-[19 Oct] Fix: a line added on 14 Oct sat in the wrong handler, so viewing an MRF request (GET /api/mrf/:id) always failed and editing a budget did not refresh JD results. Fixed with section E. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
+    <t>E. CEO clarity, dashboard &amp; analytics</t>
+  </si>
+  <si>
+    <t>N35 · Labels &amp; legends</t>
+  </si>
+  <si>
+    <t>Today: The CEO couldn't tell what pipeline columns and statuses mean. "Invited" actually means the Zeko link was sent and "In progress" means not yet invited (explained the other way round in the demo). The board doesn't show whether an Evalground test was sent.
+Change: Clear stage / status names and a legend on the pipeline board; "Test sent - due date / Overdue" on Evalground cards; review other unclear labels (screening match chips, upload job statuses) and add tooltips.
+Done when: Someone new can read the board without explanation.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 3 Enh. rows 3-4).
+[19 Oct] Built: plain card labels (Not yet invited / Zeko link sent / Not yet scheduled / Awaiting action / Awaiting decision / Test not sent / Test sent · due &lt;date&gt; / Test overdue) with hover text; a "What do these mean?" legend on the board; stage meanings on column headers; clearer labels and tooltips on Screening chips, upload statuses, MRF badges and the Vendor dashboard. Tested on staging data: labels, legend and assessment cards pass (e2e/section-e.spec.js). Final wording to confirm with RT. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
+  </si>
+  <si>
+    <t>N36 · Dashboard fixes</t>
+  </si>
+  <si>
+    <t>Today: Trends and top roles use only the newest 200 candidates; Shortlisted / Hired counts use old status values; Upcoming Interviews shows only Zeko windows (no Teams interviews) and opens Analytics; recent uploads don't open the candidate; the role filter uses the candidate's typed "Position Applied".
+Change: Server-side totals; counts aligned with pipeline statuses; Teams interviews included; rows open the right candidate; role filter by MRF; clear shortlist-rate definition.
+Done when: Dashboard numbers match Analytics and Search Candidate for the same period.</t>
+  </si>
+  <si>
+    <t>Our #61; 10 Sep dashboard-numbers item.
+[19 Oct] Built: dashboard counts every candidate on the server (no 200 cap); Shortlisted = in the pipeline now, Hired = the Analytics rule; working MRF filter; Zeko + Teams in Upcoming Interviews; rows open the candidate; "Definitions updated" note. Tested on staging data: matches Analytics for 7/30/90 days and per MRF (check-dashboard-vs-analytics.mjs all OK); filters and links pass on screen. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
+  </si>
+  <si>
+    <t>N37 · Raw vs qualified (interim)</t>
+  </si>
+  <si>
+    <t>Today: There is no view of raw vs qualified candidate numbers.
+Change: Two numbers from existing data: raw (all candidates in the period) and qualified (completed the details form or replied). Definition agreed with Chhaya first.
+Done when: Both numbers show on the dashboard, with the definition in a tooltip.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 3 Enh. row 2). The stored status is Responded status &amp; source marker (P01).
+[19 Oct] On hold until Chhaya agrees the definition. Proposed: raw = candidates added in the period; qualified = those who completed the details form or replied by email. Totals only until JD tagging (N13). About 6 h once agreed.</t>
+  </si>
+  <si>
+    <t>N38 · Recency filter</t>
+  </si>
+  <si>
+    <t>Today: Screening can't be limited to recent candidates, and the ranking doesn't use dates.
+Change: "Added in" filter: last 7 / 10 / 15 days, 1 month, 3 months.
+Done when: The filter works in both keyword and JD screening.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 4 sheet row 84). Dates in the ranking are Scoring weights &amp; recency (L01).
+[19 Oct] Built: "Added within" 7 / 10 / 15 days, 1 month, 3 months on Keyword and JD screening; the JD CSV follows the filter. Tested on staging data: JD integration 13/13 incl. the 15-day case; both filters pass on screen. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
+  </si>
+  <si>
+    <t>N39 · Analytics - Positions tab</t>
+  </si>
+  <si>
+    <t>Today: Analytics shows one MRF at a time; there is no cross-position view, no open-to-close journey and no joining ratio.
+Change: New tab with one row per MRF: opened, days open, shortlisted, candidates per stage, offers, joined, closed and reason; hiring-to-joining ratio; per-role "Moved Forward".
+Done when: Every position's status is visible on one screen.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 3 Enh. row 5); Anuj in the demo.
+[19 Oct] Built: Analytics "Positions" tab, one row per MRF (opened, days open, per-stage counts, offers, joined, joining ratio, closure reason), sortable, CSV, a row opens that MRF's funnel. Tested on staging data: rows, sort, filter, CSV and row-to-funnel pass. Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-19-phase3-section-e.md</t>
+  </si>
+  <si>
+    <t>F. Developer logging &amp; system documentation</t>
+  </si>
+  <si>
+    <t>N42 · Developer logging &amp; error tracing</t>
+  </si>
+  <si>
+    <t>Today: Developers hear about problems from HR. Logs are files on the server, and nothing ties an HR report to a log line. Scheduled-job failures and crashes are only logged, and browser errors aren't captured.
+Change: A reference ID on every request, shown in error messages ("ref: AB12CD"); logging of calls to Graph, Zeko, the AI service and Cohere; alerts on job failures and crashes; browser error capture; an admin "Logs &amp; errors" page searchable by reference, user and time; a deep health check. Personal data is masked in all logs.
+Done when: HR quotes the error reference shown on screen, and a developer finds the full trail in under 2 minutes without logging in to the server.</t>
+  </si>
+  <si>
+    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.</t>
+  </si>
+  <si>
+    <t>N43 · System documentation &amp; development history</t>
+  </si>
+  <si>
+    <t>Today: Knowledge is spread across 50+ feature plans, RCAs and changelogs. Nothing describes how the system works as a whole, what has been built since January, or how to handle common incidents.
+Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it.
+Done when: A developer new to the project can set up, find any module, handle a common incident, and see what was built, when and why, from these docs alone.</t>
+  </si>
+  <si>
+    <t>Week 4-5</t>
+  </si>
+  <si>
+    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.</t>
+  </si>
+  <si>
+    <t>G. Housekeeping (no code)</t>
+  </si>
+  <si>
+    <t>N40 · Housekeeping</t>
+  </si>
+  <si>
+    <t>Today: Stale / test MRFs (e.g. Business Development Services, T Snap Project One) show as open; Samriddhi is tagged to the wrong JD; HRD (Susmita, Subhajit) run some hiring outside the ATS.
+Change: Close the stale MRFs with a reason; close Samriddhi's wrong journey; create ATS logins with upload access for Susmita and Subhajit (role and modules set by the admin).
+Done when: The open-positions list is accurate and HRD candidates are entered in the ATS.</t>
+  </si>
+  <si>
+    <t>Demo 28 Sep. Admin action.
+[15 Oct] Admin action, not done yet. Steps in docs/changelog/CHANGES-2026-10-14-phase3-week1.md (release step 9).</t>
+  </si>
+  <si>
+    <t>H. To brainstorm later</t>
+  </si>
+  <si>
+    <t>N41 · Upload speed</t>
+  </si>
+  <si>
+    <t>Today: RT reports that uploads take too long; each resume or Excel row is parsed by AI one at a time, followed by more AI work per candidate.
+Change: To be decided in a separate brainstorm once all other Do Now items are closed.
+Done when: -</t>
+  </si>
+  <si>
+    <t>Brainstorm later</t>
+  </si>
+  <si>
+    <t>After other items</t>
+  </si>
+  <si>
+    <t>RT "Matching &amp; score analysis takes too long to upload".</t>
+  </si>
+  <si>
+    <t>Search, scoring &amp; candidate movement</t>
+  </si>
+  <si>
+    <t>L01 · Scoring weights &amp; recency</t>
+  </si>
+  <si>
+    <t>Today: After JD - skill gate through JD - ranking (N07–N09), ranking among qualified candidates uses fixed weights and ignores when a candidate applied.
+Change: Re-tune weights and score bands with RT; rank recent applicants higher.
+Done when: RT agrees with the ranking on their sample JDs.</t>
+  </si>
+  <si>
+    <t>RT §5; CEO (Phase 4 sheet row 84).</t>
+  </si>
+  <si>
+    <t>L02 · Move / re-tag candidate</t>
+  </si>
+  <si>
+    <t>Today: A candidate already tagged to one JD can't be moved to another; a wrong tag can only be closed; tags always start at the first stage.
+Change: Move a candidate to another JD with a chosen landing stage (history kept); remove a wrong tag.
+Done when: A final-round candidate can move to a new role at a chosen stage without extra emails.</t>
+  </si>
+  <si>
+    <t>RT §6.2. Needs RT's decision on where a moved candidate lands.</t>
+  </si>
+  <si>
+    <t>L03 · Flexible stages</t>
+  </si>
+  <si>
+    <t>Today: The pipeline moves forward one stage at a time; only Tech 3 and the Client round can be skipped; a skipped stage can never be done later.
+Change: Authorized users can skip stages (e.g. HR Screening -&gt; Evalground, HR Screening -&gt; Functional, Assessment -&gt; CEO round) and re-open or complete a skipped stage later (walk-in: Tech 1 first, Evalground at the weekend). Evalground import matches candidates at any stage; candidates get no duplicate emails.
+Done when: The walk-in example runs end to end with correct emails and history.</t>
+  </si>
+  <si>
+    <t>RT §7. Needs written answers: who may skip, and what the candidate is told.</t>
+  </si>
+  <si>
+    <t>MRF &amp; pipeline hygiene</t>
+  </si>
+  <si>
+    <t>L04 · MRF Hold</t>
+  </si>
+  <si>
+    <t>Today: Approvers can only approve or reject an MRF.
+Change: Hold option (with a note and hold-until date) at approval; on that date the approver is reminded with Approve / Reject / Hold further; held MRFs appear as open nowhere.
+Done when: A held MRF re-prompts its approver on the hold-until date.</t>
+  </si>
+  <si>
+    <t>RT §1.</t>
+  </si>
+  <si>
+    <t>L05 · Drop-out rules</t>
+  </si>
+  <si>
+    <t>Today: Candidates who never take a Zeko test or respond stay in the pipeline indefinitely and clutter the columns.
+Change: Per-stage reminder and timeout rules; auto-close as "Unresponsive" after the timeout; settings to tune them.
+Done when: Non-responders leave the board automatically after the set time.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 4 sheet row 85). Needs RT sign-off (current rule: recruiter decides).</t>
+  </si>
+  <si>
+    <t>Analytics &amp; JD records</t>
+  </si>
+  <si>
+    <t>L06 · Analytics - date range &amp; Total Applied</t>
+  </si>
+  <si>
+    <t>Today: Analytics uses fixed windows, and "Total Applied" per role can't be counted without JD tags.
+Change: Presets (30 / 60 / 90 / 365 days, all) plus a custom date picker applied to every tile; per-role "Total Applied" from the JD tags (JD tagging on upload (N13–N15)).
+Done when: Every Analytics number follows the chosen range.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 3 Enh. row 5); 10 Sep review.</t>
+  </si>
+  <si>
+    <t>L07 · Editable JD label (no MRF)</t>
+  </si>
+  <si>
+    <t>Today: JDs without an MRF have no date or label to tell versions apart.
+Change: Recruiter-editable date / label on such JDs, shown next to the JD name.
+Done when: RT can mark the latest version of a JD that has no MRF.</t>
+  </si>
+  <si>
+    <t>RT §3 (second half).</t>
+  </si>
+  <si>
+    <t>Other Bugs</t>
+  </si>
+  <si>
+    <t>Adhoc links for all forms</t>
+  </si>
+  <si>
+    <t>If Recruiter wants to access some links, right now, they are not accessible easily. Let's say I have sent a link to interviewer post interview, I can't find the link form the app easily. There are lot more forms and lot more links. If we can arrange those links in some page, it would make things easier for recruiter for fetch any link</t>
+  </si>
+  <si>
+    <t>HR Manual Upload &amp; Vendor Manual Upload</t>
+  </si>
+  <si>
+    <t>If there is any duplicate, right now,REVIEW is showing what is the current user name and his/her resume instead of a pure comparison of what data has been there already vs what is new one and what changed since last resume etc.</t>
+  </si>
+  <si>
+    <t>HR Manual Upload - User Profile redirect</t>
+  </si>
+  <si>
+    <t>In the resume uploaded by HR, if user wants to check the candidate details in detail, they don't have the option to redirect the user to the candidate profile view page.</t>
+  </si>
+  <si>
+    <t>Candidate Screening - Hidden by system data</t>
+  </si>
+  <si>
+    <t>For example - "8 recently rejected for this role · 3 meet education, budget and experience · of those, 0 have all 7 mandatory skills
+" for this case, if I wish to see the data, there is no such option exist now.</t>
+  </si>
+  <si>
+    <t>Dossier Enhancements</t>
+  </si>
+  <si>
+    <t>1. dossier was giving details in horizontal, also edited tech 1 feedback was not added here.can we make this vericle, it will be easy to read</t>
+  </si>
+  <si>
+    <t>Meetings links</t>
+  </si>
+  <si>
+    <t>A link to the meeting should be avaiable for non ats persons too (if i copy the link from ATS share the recording of interview outside ATS via outlook mail will mam be able to access it.)</t>
+  </si>
+  <si>
+    <t>Report link for the next round</t>
+  </si>
+  <si>
+    <t>When tech1 round done and passed, when we are about to schedule round 2, all the details of round 1 score, recording and cv should be sharing to the tech2 round interviewer only. (t tech 2 interviewer when we schedule can get tech 1 scorecard report, similarly tech 3 or HR can get cumulative report, also do we receive notification once someone submit feedback on recruitment id.)</t>
+  </si>
+  <si>
+    <t>Vendor 2 - C2C Vendor (on hold)</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. NULL vendor_type = placement backward-compatible</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months.</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Keeps shared tracking/status steps single-sourced</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Rate/Duration required for C2C optional for placement</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Shared engine reused - not a fork of the 1724-line runBatchParsing</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Flags already_in_main_pool - never auto-merges/rejects</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Name collision in C2C is expected not an error</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Review never vendor-accessible</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Never mutate the raw Name field</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Education + stability weights zeroed for C2C</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Reuses existing premium upload components</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. No UNION logic needed in controller</t>
+  </si>
+  <si>
+    <t>On hold - per Sanghamitra, until the core runs stable for 1-2 months. Proves the shared engine was not regressed</t>
+  </si>
+  <si>
+    <t>MS Access (R&amp;D / export)</t>
+  </si>
+  <si>
+    <t>Other Phase 4 items</t>
+  </si>
+  <si>
+    <t>P01 · Responded status &amp; source marker</t>
+  </si>
+  <si>
+    <t>Today: Nothing records whether a candidate responded to outreach or is an old database record, so search can't prefer active applicants.
+Change: Store the responded status and source (new applicant vs old database); rank late responders lower; "Responders only" option in search; the Raw vs qualified (interim) (N37) counts switch to the stored status.
+Done when: Search can be limited to responders, and each card shows "Responded" or "From old database".</t>
+  </si>
+  <si>
+    <t>CEO (Phase 3 Enh. row 2; Phase 4 sheet row 83).</t>
+  </si>
+  <si>
+    <t>P02 · Hiring-manager status email</t>
+  </si>
+  <si>
+    <t>Today: RT sends daily / weekly position updates to hiring managers by hand.
+Change: Automatic daily or weekly email to each hiring manager about their open positions (candidates per stage, upcoming interviews, offers); schedule set in Settings.
+Done when: Hiring managers receive it without RT's involvement.</t>
+  </si>
+  <si>
+    <t>Anuj in the demo; our #71.</t>
+  </si>
+  <si>
+    <t>P03 · Hiring-manager read-only role</t>
+  </si>
+  <si>
+    <t>Today: Hiring managers have no ATS login.
+Change: A read-only role that sees only the hiring manager's own positions (pipeline and analytics).
+Done when: A hiring manager logs in and sees only their positions, with no edit actions.</t>
+  </si>
+  <si>
+    <t>CEO (Phase 4 sheet row 86). Hiring-manager status email (P02) covers the status need first.</t>
+  </si>
+  <si>
+    <t>P04 · SMS / WhatsApp reminders</t>
+  </si>
+  <si>
+    <t>Today: The ATS can only send email.
+Change: Interview reminders by SMS / WhatsApp through a provider, using the phone captured in Candidate phone &amp; interview reminders (N22).
+Done when: A scheduled interview triggers an SMS / WhatsApp reminder.</t>
+  </si>
+  <si>
+    <t>RT §9. Needs a provider.</t>
+  </si>
+  <si>
+    <t>P05 · Prompt configuration</t>
+  </si>
+  <si>
+    <t>Today: All six AI prompts (JD parse, resume parse, two insight prompts, two Evalground prompts) are hard-coded.
+Change: Admin screen to view and edit prompts, with versioning, reset to default and a test run.
+Done when: A prompt can be changed and rolled back without a deployment.</t>
+  </si>
+  <si>
+    <t>Our list.</t>
+  </si>
+  <si>
+    <t>P06 · Reminder settings in one place</t>
+  </si>
+  <si>
+    <t>Today: Settings &gt; Reminder Settings covers only three reminder types; interview, occurrence, document and assessment reminders are set elsewhere or in server config.
+Change: Bring every reminder's on/off switch, timing and limits under one Settings section.
+Done when: All reminders can be tuned from Settings.</t>
+  </si>
+  <si>
+    <t>P07 · Website candidates report</t>
+  </si>
+  <si>
+    <t>Today: Website applications reach the ATS through the recruitment mailbox but aren't marked as website-sourced, and RT has no daily report of them.
+Change: Store a permanent intake source on each candidate; daily 8 AM email to RT with the current month's website candidates as Excel; on the 1st, a second email with the previous month's summary.
+Done when: RT receives both emails on schedule.</t>
+  </si>
+  <si>
+    <t>Our list (Website Data Update; Website Integration).</t>
+  </si>
+  <si>
+    <t>P08 · Captcha on public MRF form</t>
+  </si>
+  <si>
+    <t>Today: Captcha protects the login pages, but the public MRF submission form has no captcha or rate limit.
+Change: Add captcha and a rate limit to the public MRF form.
+Done when: Automated submissions are blocked.</t>
+  </si>
+  <si>
+    <t>Our list (Captcha).</t>
+  </si>
+  <si>
+    <t>P09 · Zeko 90-day re-interview check</t>
+  </si>
+  <si>
+    <t>Today: Nothing stops a Zeko interview being sent again to a candidate interviewed in the last 90 days.
+Change: Warn or block re-sending within 90 days and reuse the previous result; investigate whether Zeko's API allows archiving or deleting old interview data.
+Done when: Re-sending within 90 days shows a warning with the previous result.</t>
+  </si>
+  <si>
+    <t>Our list (R&amp;D). Hours exclude the Zeko API research.</t>
+  </si>
+  <si>
+    <t>P10 · Admin Config UI polish</t>
+  </si>
+  <si>
+    <t>Today: Admins can edit stages, outcomes and reasons, but there is no hard delete, no in-use check when deactivating outcomes or reasons, no audit of config changes, and new custom interview stages get no scheduling or scorecards.
+Change: Add those four.
+Done when: Config changes are logged and can't break candidates mid-stage.</t>
+  </si>
+  <si>
+    <t>P11 · Excel scores to round scorecards</t>
+  </si>
+  <si>
+    <t>Today: Interview scores in Excel uploads are stored on the candidate record, not in the round scorecards the pipeline uses (Scores in the pipeline drawer (N28) only displays them).
+Change: Import them into the matching round's scorecard.
+Done when: Uploaded scores appear as real round scores.</t>
+  </si>
+  <si>
+    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.
+[20 Oct] Built: error ref on every request ("ref: K7Q2MX" on server errors), masked logs, every outside call logged, error store rpa_error_log (DDL 2026-10-20-error-log.sql, applied on staging 20 Oct; kept 30 days), alerts and heartbeats for all scheduled jobs, crash alerts, browser error capture, Super Admin → Logs &amp; errors (Errors, Find a ref, Jobs, Health). Tested on the staging DB: unit 20/20, integration 6/6, forced job failure → one alert, Logs &amp; errors endpoints checked (Health all green). Screens not checked in the browser (no Super Admin login). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
+  </si>
+  <si>
+    <t>Today: Knowledge is spread across 50+ feature plans, RCAs and changelogs. Nothing describes how the system works as a whole, what has been built since January, or how to handle common incidents.
+Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it. Plus step-by-step user guides for HR/recruiters, Admins, Super Admins, vendors and email-only users (docs/user-guides/), added 19 Oct.
+Done when: A developer new to the project can set up, find any module, handle a common incident, and see what was built, when and why, from these docs alone.</t>
+  </si>
+  <si>
+    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.
+[20 Oct] Written: docs/system/ (8 developer pages incl. operations runbook and 2026 development history), a root README, and business user guides in docs/user-guides/ (Recruiter &amp; HR with masked screenshots, Admin, Super Admin, Vendor, email-only users). Scope grew 24 → 44 h with the user guides (decision 19 Oct). Review pending (Harish; Pankaj and RT dry runs). Admin / Super Admin screenshots need a Super Admin login. PDFs exported at release. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
   </si>
 </sst>
 </file>
@@ -4821,12 +4809,12 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -17575,7 +17563,7 @@
         <v>938</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>1174</v>
+        <v>960</v>
       </c>
       <c r="J10" s="4"/>
     </row>
@@ -18277,7 +18265,7 @@
         <v>772</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>1170</v>
+        <v>1032</v>
       </c>
       <c r="J35" s="4"/>
     </row>
@@ -18307,7 +18295,7 @@
         <v>772</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>1171</v>
+        <v>1035</v>
       </c>
       <c r="J36" s="4"/>
     </row>
@@ -18397,7 +18385,7 @@
         <v>768</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>1172</v>
+        <v>1044</v>
       </c>
       <c r="J39" s="4"/>
     </row>
@@ -18457,7 +18445,7 @@
         <v>772</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>1173</v>
+        <v>1050</v>
       </c>
       <c r="J41" s="4"/>
     </row>
@@ -18501,7 +18489,7 @@
         <v>772</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>1165</v>
+        <v>1054</v>
       </c>
       <c r="J43" s="4"/>
     </row>
@@ -18531,7 +18519,7 @@
         <v>993</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>1166</v>
+        <v>1057</v>
       </c>
       <c r="J44" s="4"/>
     </row>
@@ -18561,7 +18549,7 @@
         <v>993</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>1167</v>
+        <v>1060</v>
       </c>
       <c r="J45" s="4"/>
     </row>
@@ -18591,7 +18579,7 @@
         <v>938</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>1168</v>
+        <v>1063</v>
       </c>
       <c r="J46" s="4"/>
     </row>
@@ -18621,7 +18609,7 @@
         <v>993</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>1169</v>
+        <v>1066</v>
       </c>
       <c r="J47" s="4"/>
     </row>
@@ -18650,10 +18638,10 @@
         <v>82</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>31</v>
+        <v>341</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>34</v>
+        <v>709</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>226</v>
@@ -18665,7 +18653,7 @@
         <v>772</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>1070</v>
+        <v>1170</v>
       </c>
       <c r="J49" s="4"/>
     </row>
@@ -18674,28 +18662,28 @@
         <v>1071</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>1072</v>
+        <v>1171</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>82</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>31</v>
+        <v>341</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>34</v>
+        <v>709</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>226</v>
       </c>
       <c r="G50" s="4">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="H50" s="4" t="s">
         <v>1073</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>1074</v>
+        <v>1172</v>
       </c>
       <c r="J50" s="4"/>
     </row>
@@ -18807,7 +18795,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -19185,13 +19173,32 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
-      <c r="B17" t="s">
+    <row r="17" ht="27.6" spans="1:2">
+      <c r="A17" t="s">
         <v>1118</v>
       </c>
+      <c r="B17" s="6" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1123</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J17" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:J19" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <mergeCells count="4">
@@ -19256,7 +19263,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>1119</v>
+        <v>1124</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -19292,7 +19299,7 @@
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
-        <v>1120</v>
+        <v>1125</v>
       </c>
       <c r="J3" s="4"/>
     </row>
@@ -19320,7 +19327,7 @@
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J4" s="4"/>
     </row>
@@ -19348,7 +19355,7 @@
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J5" s="4"/>
     </row>
@@ -19376,7 +19383,7 @@
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J6" s="4"/>
     </row>
@@ -19404,7 +19411,7 @@
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4" t="s">
-        <v>1122</v>
+        <v>1127</v>
       </c>
       <c r="J7" s="4"/>
     </row>
@@ -19432,7 +19439,7 @@
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J8" s="4"/>
     </row>
@@ -19460,7 +19467,7 @@
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J9" s="4"/>
     </row>
@@ -19488,7 +19495,7 @@
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J10" s="4"/>
     </row>
@@ -19516,7 +19523,7 @@
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J11" s="4"/>
     </row>
@@ -19544,7 +19551,7 @@
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4" t="s">
-        <v>1123</v>
+        <v>1128</v>
       </c>
       <c r="J12" s="4"/>
     </row>
@@ -19572,7 +19579,7 @@
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J13" s="4"/>
     </row>
@@ -19600,7 +19607,7 @@
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="4" t="s">
-        <v>1124</v>
+        <v>1129</v>
       </c>
       <c r="J14" s="4"/>
     </row>
@@ -19628,7 +19635,7 @@
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>1125</v>
+        <v>1130</v>
       </c>
       <c r="J15" s="4"/>
     </row>
@@ -19656,7 +19663,7 @@
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J16" s="4"/>
     </row>
@@ -19684,7 +19691,7 @@
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J17" s="4"/>
     </row>
@@ -19712,7 +19719,7 @@
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J18" s="4"/>
     </row>
@@ -19740,7 +19747,7 @@
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J19" s="4"/>
     </row>
@@ -19768,7 +19775,7 @@
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J20" s="4"/>
     </row>
@@ -19796,7 +19803,7 @@
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J21" s="4"/>
     </row>
@@ -19824,7 +19831,7 @@
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4" t="s">
-        <v>1126</v>
+        <v>1131</v>
       </c>
       <c r="J22" s="4"/>
     </row>
@@ -19852,7 +19859,7 @@
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4" t="s">
-        <v>1127</v>
+        <v>1132</v>
       </c>
       <c r="J23" s="4"/>
     </row>
@@ -19880,7 +19887,7 @@
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="4" t="s">
-        <v>1128</v>
+        <v>1133</v>
       </c>
       <c r="J24" s="4"/>
     </row>
@@ -19908,7 +19915,7 @@
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4" t="s">
-        <v>1129</v>
+        <v>1134</v>
       </c>
       <c r="J25" s="4"/>
     </row>
@@ -19936,7 +19943,7 @@
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J26" s="4"/>
     </row>
@@ -19964,7 +19971,7 @@
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J27" s="4"/>
     </row>
@@ -19992,7 +19999,7 @@
       </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4" t="s">
-        <v>1130</v>
+        <v>1135</v>
       </c>
       <c r="J28" s="4"/>
     </row>
@@ -20020,7 +20027,7 @@
       </c>
       <c r="H29" s="4"/>
       <c r="I29" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J29" s="4"/>
     </row>
@@ -20048,7 +20055,7 @@
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J30" s="4"/>
     </row>
@@ -20076,7 +20083,7 @@
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4" t="s">
-        <v>1131</v>
+        <v>1136</v>
       </c>
       <c r="J31" s="4"/>
     </row>
@@ -20104,7 +20111,7 @@
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J32" s="4"/>
     </row>
@@ -20132,7 +20139,7 @@
       </c>
       <c r="H33" s="4"/>
       <c r="I33" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J33" s="4"/>
     </row>
@@ -20160,7 +20167,7 @@
       </c>
       <c r="H34" s="4"/>
       <c r="I34" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J34" s="4"/>
     </row>
@@ -20188,7 +20195,7 @@
       </c>
       <c r="H35" s="4"/>
       <c r="I35" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J35" s="4"/>
     </row>
@@ -20216,7 +20223,7 @@
       </c>
       <c r="H36" s="4"/>
       <c r="I36" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J36" s="4"/>
     </row>
@@ -20244,7 +20251,7 @@
       </c>
       <c r="H37" s="4"/>
       <c r="I37" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J37" s="4"/>
     </row>
@@ -20272,7 +20279,7 @@
       </c>
       <c r="H38" s="4"/>
       <c r="I38" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J38" s="4"/>
     </row>
@@ -20300,7 +20307,7 @@
       </c>
       <c r="H39" s="4"/>
       <c r="I39" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J39" s="4"/>
     </row>
@@ -20328,7 +20335,7 @@
       </c>
       <c r="H40" s="4"/>
       <c r="I40" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J40" s="4"/>
     </row>
@@ -20356,7 +20363,7 @@
       </c>
       <c r="H41" s="4"/>
       <c r="I41" s="4" t="s">
-        <v>1132</v>
+        <v>1137</v>
       </c>
       <c r="J41" s="4"/>
     </row>
@@ -20384,13 +20391,13 @@
       </c>
       <c r="H42" s="4"/>
       <c r="I42" s="4" t="s">
-        <v>1121</v>
+        <v>1126</v>
       </c>
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="2" t="s">
-        <v>1133</v>
+        <v>1138</v>
       </c>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -20512,7 +20519,7 @@
     </row>
     <row r="48" spans="1:10">
       <c r="A48" s="2" t="s">
-        <v>1134</v>
+        <v>1139</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -20526,10 +20533,10 @@
     </row>
     <row r="49" ht="106.5" customHeight="1" spans="1:10">
       <c r="A49" s="4" t="s">
-        <v>1135</v>
+        <v>1140</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>1136</v>
+        <v>1141</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>126</v>
@@ -20548,16 +20555,16 @@
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="4" t="s">
-        <v>1137</v>
+        <v>1142</v>
       </c>
       <c r="J49" s="4"/>
     </row>
     <row r="50" ht="76.5" customHeight="1" spans="1:10">
       <c r="A50" s="4" t="s">
-        <v>1138</v>
+        <v>1143</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>1139</v>
+        <v>1144</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>106</v>
@@ -20576,16 +20583,16 @@
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4" t="s">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="J50" s="4"/>
     </row>
     <row r="51" ht="76.5" customHeight="1" spans="1:10">
       <c r="A51" s="4" t="s">
-        <v>1141</v>
+        <v>1146</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>1142</v>
+        <v>1147</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>126</v>
@@ -20604,16 +20611,16 @@
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>1143</v>
+        <v>1148</v>
       </c>
       <c r="J51" s="4"/>
     </row>
     <row r="52" ht="61.5" customHeight="1" spans="1:10">
       <c r="A52" s="4" t="s">
-        <v>1144</v>
+        <v>1149</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>1145</v>
+        <v>1150</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>126</v>
@@ -20632,16 +20639,16 @@
       </c>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>1146</v>
+        <v>1151</v>
       </c>
       <c r="J52" s="4"/>
     </row>
     <row r="53" ht="76.5" customHeight="1" spans="1:10">
       <c r="A53" s="4" t="s">
-        <v>1147</v>
+        <v>1152</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>1148</v>
+        <v>1153</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>106</v>
@@ -20660,16 +20667,16 @@
       </c>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" ht="91.5" customHeight="1" spans="1:10">
       <c r="A54" s="4" t="s">
-        <v>1150</v>
+        <v>1155</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>1151</v>
+        <v>1156</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>106</v>
@@ -20688,16 +20695,16 @@
       </c>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="J54" s="4"/>
     </row>
     <row r="55" ht="91.5" customHeight="1" spans="1:10">
       <c r="A55" s="4" t="s">
-        <v>1152</v>
+        <v>1157</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>1153</v>
+        <v>1158</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>106</v>
@@ -20716,16 +20723,16 @@
       </c>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>1154</v>
+        <v>1159</v>
       </c>
       <c r="J55" s="4"/>
     </row>
     <row r="56" ht="61.5" customHeight="1" spans="1:10">
       <c r="A56" s="4" t="s">
-        <v>1155</v>
+        <v>1160</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>1156</v>
+        <v>1161</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>106</v>
@@ -20744,16 +20751,16 @@
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>1157</v>
+        <v>1162</v>
       </c>
       <c r="J56" s="4"/>
     </row>
     <row r="57" ht="106.5" customHeight="1" spans="1:10">
       <c r="A57" s="4" t="s">
-        <v>1158</v>
+        <v>1163</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>1159</v>
+        <v>1164</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>106</v>
@@ -20772,16 +20779,16 @@
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
-        <v>1160</v>
+        <v>1165</v>
       </c>
       <c r="J57" s="4"/>
     </row>
     <row r="58" ht="76.5" customHeight="1" spans="1:10">
       <c r="A58" s="4" t="s">
-        <v>1161</v>
+        <v>1166</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>1162</v>
+        <v>1167</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>106</v>
@@ -20800,16 +20807,16 @@
       </c>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="J58" s="4"/>
     </row>
     <row r="59" ht="76.5" customHeight="1" spans="1:10">
       <c r="A59" s="4" t="s">
-        <v>1163</v>
+        <v>1168</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>1164</v>
+        <v>1169</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>106</v>
@@ -20828,7 +20835,7 @@
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
-        <v>1149</v>
+        <v>1154</v>
       </c>
       <c r="J59" s="4"/>
     </row>
@@ -21716,7 +21723,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="J28:J31 J46 J36 J39:J43 J71:J1048576 J48:J69" listDataValidation="1"/>
+    <ignoredError sqref="J48:J69 J71:J1048576 J39:J43 J36 J46 J28:J31" listDataValidation="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Development of B- JD tagging on upload, G - Housekeeping, and H - To brainstorm later
</commit_message>
<xml_diff>
--- a/docs/Phase 3 Enhancements or Feedback/ATS App - Phase wise Task Items.xlsx
+++ b/docs/Phase 3 Enhancements or Feedback/ATS App - Phase wise Task Items.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4789" uniqueCount="1173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4789" uniqueCount="1170">
   <si>
     <t>Task</t>
   </si>
@@ -4139,21 +4139,23 @@
 Done when: HR quotes the error reference shown on screen, and a developer finds the full trail in under 2 minutes without logging in to the server.</t>
   </si>
   <si>
-    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.</t>
+    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.
+[20 Oct] Built: error ref on every request ("ref: K7Q2MX" on server errors), masked logs, every outside call logged, error store rpa_error_log (DDL 2026-10-20-error-log.sql, applied on staging 20 Oct; kept 30 days), alerts and heartbeats for all scheduled jobs, crash alerts, browser error capture, Super Admin → Logs &amp; errors (Errors, Find a ref, Jobs, Health). Tested on the staging DB: unit 20/20, integration 6/6, forced job failure → one alert, Logs &amp; errors endpoints checked (Health all green). Screens not checked in the browser (no Super Admin login). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
   </si>
   <si>
     <t>N43 · System documentation &amp; development history</t>
   </si>
   <si>
     <t>Today: Knowledge is spread across 50+ feature plans, RCAs and changelogs. Nothing describes how the system works as a whole, what has been built since January, or how to handle common incidents.
-Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it.
+Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it. Plus step-by-step user guides for HR/recruiters, Admins, Super Admins, vendors and email-only users (docs/user-guides/), added 19 Oct.
 Done when: A developer new to the project can set up, find any module, handle a common incident, and see what was built, when and why, from these docs alone.</t>
   </si>
   <si>
     <t>Week 4-5</t>
   </si>
   <si>
-    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.</t>
+    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.
+[20 Oct] Written: docs/system/ (8 developer pages incl. operations runbook and 2026 development history), a root README, and business user guides in docs/user-guides/ (Recruiter &amp; HR with masked screenshots, Admin, Super Admin, Vendor, email-only users). Scope grew 24 → 44 h with the user guides (decision 19 Oct). Review pending (Harish; Pankaj and RT dry runs). Admin / Super Admin screenshots need a Super Admin login. PDFs exported at release. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
   </si>
   <si>
     <t>G. Housekeeping (no code)</t>
@@ -4481,19 +4483,6 @@
     <t>Today: Interview scores in Excel uploads are stored on the candidate record, not in the round scorecards the pipeline uses (Scores in the pipeline drawer (N28) only displays them).
 Change: Import them into the matching round's scorecard.
 Done when: Uploaded scores appear as real round scores.</t>
-  </si>
-  <si>
-    <t>Our #52 ("logs should be visible to developers"); CEO (Phase 3 Enh. row 6). Replaces the parked longevity alerts and error view items.
-[20 Oct] Built: error ref on every request ("ref: K7Q2MX" on server errors), masked logs, every outside call logged, error store rpa_error_log (DDL 2026-10-20-error-log.sql, applied on staging 20 Oct; kept 30 days), alerts and heartbeats for all scheduled jobs, crash alerts, browser error capture, Super Admin → Logs &amp; errors (Errors, Find a ref, Jobs, Health). Tested on the staging DB: unit 20/20, integration 6/6, forced job failure → one alert, Logs &amp; errors endpoints checked (Health all green). Screens not checked in the browser (no Super Admin login). Not yet deployed to staging. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
-  </si>
-  <si>
-    <t>Today: Knowledge is spread across 50+ feature plans, RCAs and changelogs. Nothing describes how the system works as a whole, what has been built since January, or how to handle common incidents.
-Change: A docs/system/ set covering overview and architecture, modules, data model, jobs and integrations, configuration, an operations runbook, onboarding, and a development history from January 2026 (the n8n phases, the move to full stack in June, Phase 2 and Phase 3). Each release then updates it. Plus step-by-step user guides for HR/recruiters, Admins, Super Admins, vendors and email-only users (docs/user-guides/), added 19 Oct.
-Done when: A developer new to the project can set up, find any module, handle a common incident, and see what was built, when and why, from these docs alone.</t>
-  </si>
-  <si>
-    <t>Your request; CEO (Phase 3 Enh. row 6). Replaces the parked longevity runbook item.
-[20 Oct] Written: docs/system/ (8 developer pages incl. operations runbook and 2026 development history), a root README, and business user guides in docs/user-guides/ (Recruiter &amp; HR with masked screenshots, Admin, Super Admin, Vendor, email-only users). Scope grew 24 → 44 h with the user guides (decision 19 Oct). Review pending (Harish; Pankaj and RT dry runs). Admin / Super Admin screenshots need a Super Admin login. PDFs exported at release. Where: docs/changelog/CHANGES-2026-10-20-phase3-section-f.md</t>
   </si>
 </sst>
 </file>
@@ -4809,12 +4798,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="134"/>
@@ -18653,7 +18642,7 @@
         <v>772</v>
       </c>
       <c r="I49" s="4" t="s">
-        <v>1170</v>
+        <v>1070</v>
       </c>
       <c r="J49" s="4"/>
     </row>
@@ -18662,7 +18651,7 @@
         <v>1071</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>1171</v>
+        <v>1072</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>82</v>
@@ -18683,7 +18672,7 @@
         <v>1073</v>
       </c>
       <c r="I50" s="4" t="s">
-        <v>1172</v>
+        <v>1074</v>
       </c>
       <c r="J50" s="4"/>
     </row>
@@ -21723,7 +21712,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="J48:J69 J71:J1048576 J39:J43 J36 J46 J28:J31" listDataValidation="1"/>
+    <ignoredError sqref="J28:J31 J46 J36 J39:J43 J71:J1048576 J48:J69" listDataValidation="1"/>
   </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>